<commit_message>
feat: add start and end time override fields to database schema
</commit_message>
<xml_diff>
--- a/outputs/2027-calendar/SwimBuddz_2027_Annual_Calendar_Reviewed.xlsx
+++ b/outputs/2027-calendar/SwimBuddz_2027_Annual_Calendar_Reviewed.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11460" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="10880"/>
   </bookViews>
   <sheets>
     <sheet name="Community" sheetId="1" r:id="rId1"/>
@@ -2537,7 +2537,7 @@
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
     </row>
-    <row r="4" customHeight="1" spans="1:8">
+    <row r="4" ht="52" customHeight="1" spans="1:8">
       <c r="A4" s="9">
         <v>46390</v>
       </c>
@@ -2617,7 +2617,7 @@
       <c r="G7" s="12"/>
       <c r="H7" s="12"/>
     </row>
-    <row r="8" ht="26.4" customHeight="1" spans="1:8">
+    <row r="8" ht="36" customHeight="1" spans="1:8">
       <c r="A8" s="9">
         <v>46394</v>
       </c>
@@ -2719,7 +2719,7 @@
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
     </row>
-    <row r="15" ht="26.4" customHeight="1" spans="1:8">
+    <row r="15" ht="36" customHeight="1" spans="1:8">
       <c r="A15" s="9">
         <v>46401</v>
       </c>

</xml_diff>